<commit_message>
Update AMD financial benchmarking Excel template formulas and input cells
Agent-Logs-Url: https://github.com/pramod51/medplus/sessions/2d9c4063-d594-41cc-a8e6-e608d662139c

Co-authored-by: ydvashwani <47135442+ydvashwani@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/financial_benchmark_template_amd.xlsx
+++ b/financial_benchmark_template_amd.xlsx
@@ -522,7 +522,7 @@
           <t>Fiscal Year</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr"/>
+      <c r="B6" s="5" t="n"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Enter reporting fiscal year (e.g., FY2025)</t>
@@ -535,7 +535,7 @@
           <t>Currency</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr"/>
+      <c r="B7" s="5" t="n"/>
       <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Enter reporting currency (e.g., USD)</t>
@@ -653,7 +653,10 @@
           <t>Total Current Assets</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
+      <c r="B17" s="6">
+        <f>B12+B14+B15+B16</f>
+        <v/>
+      </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Balance Sheet</t>
@@ -705,7 +708,10 @@
           <t>Total Current Liabilities</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n"/>
+      <c r="B21" s="6">
+        <f>B18+B19+B20</f>
+        <v/>
+      </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Balance Sheet</t>
@@ -713,17 +719,9 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Days in Year</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Manual entry (e.g., 365) for DSO calculation</t>
-        </is>
-      </c>
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
@@ -783,7 +781,7 @@
         </is>
       </c>
       <c r="B28" s="6">
-        <f>(B14/B10)*B22</f>
+        <f>(B14/B10)*365</f>
         <v/>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -799,7 +797,7 @@
         </is>
       </c>
       <c r="B29" s="6">
-        <f>B10/AVERAGE(B13,B14)</f>
+        <f>B10/((B13+B14)/2)</f>
         <v/>
       </c>
       <c r="C29" s="4" t="inlineStr">

</xml_diff>